<commit_message>
fix: harden parts fixture portability
Co-Authored-By: Paperclip <noreply@paperclip.ing>
</commit_message>
<xml_diff>
--- a/docs/testing/parts-import-fixtures/xlsx/parts-import-style-01.xlsx
+++ b/docs/testing/parts-import-fixtures/xlsx/parts-import-style-01.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="227">
   <si>
     <t>code</t>
   </si>
@@ -88,9 +88,6 @@
     <t>Bridgeport</t>
   </si>
   <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
     <t>ea</t>
   </si>
   <si>
@@ -121,12 +118,6 @@
     <t>Square D</t>
   </si>
   <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>16.97</t>
   </si>
   <si>
@@ -154,12 +145,6 @@
     <t>Raco</t>
   </si>
   <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>3.84</t>
   </si>
   <si>
@@ -187,12 +172,6 @@
     <t>Lithonia</t>
   </si>
   <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>66.83</t>
   </si>
   <si>
@@ -220,12 +199,6 @@
     <t>Leviton</t>
   </si>
   <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>4.71</t>
   </si>
   <si>
@@ -253,12 +226,6 @@
     <t>Minerallac</t>
   </si>
   <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>0.95</t>
   </si>
   <si>
@@ -286,18 +253,12 @@
     <t>Southwire</t>
   </si>
   <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
     <t>ft</t>
   </si>
   <si>
     <t>0.29</t>
   </si>
   <si>
-    <t>15</t>
-  </si>
-  <si>
     <t>23</t>
   </si>
   <si>
@@ -313,24 +274,9 @@
     <t>2 in EMT Conduit 10 ft</t>
   </si>
   <si>
-    <t>Conduit</t>
-  </si>
-  <si>
-    <t>Allied Tube</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>stick</t>
-  </si>
-  <si>
     <t>6.75</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
     <t>26</t>
   </si>
   <si>
@@ -346,24 +292,9 @@
     <t>EMT Set-Screw Connector #11</t>
   </si>
   <si>
-    <t>Fittings</t>
-  </si>
-  <si>
-    <t>Bridgeport</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>1.53</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
     <t>29</t>
   </si>
   <si>
@@ -379,24 +310,9 @@
     <t>20A 1-pole QO Plug-On Breaker</t>
   </si>
   <si>
-    <t>Breakers</t>
-  </si>
-  <si>
-    <t>Square D</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>15.93</t>
   </si>
   <si>
-    <t>24</t>
-  </si>
-  <si>
     <t>32</t>
   </si>
   <si>
@@ -412,24 +328,9 @@
     <t>Steel Device Box #1</t>
   </si>
   <si>
-    <t>Boxes</t>
-  </si>
-  <si>
-    <t>Raco</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>3.61</t>
   </si>
   <si>
-    <t>27</t>
-  </si>
-  <si>
     <t>35</t>
   </si>
   <si>
@@ -445,24 +346,9 @@
     <t>LED Flat Panel #2</t>
   </si>
   <si>
-    <t>Lighting</t>
-  </si>
-  <si>
-    <t>Lithonia</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>63.18</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
     <t>38</t>
   </si>
   <si>
@@ -478,24 +364,9 @@
     <t>Decorator Receptacle #3</t>
   </si>
   <si>
-    <t>Devices</t>
-  </si>
-  <si>
-    <t>Leviton</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>4.47</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
     <t>41</t>
   </si>
   <si>
@@ -511,24 +382,9 @@
     <t>Strut Strap #4</t>
   </si>
   <si>
-    <t>Fasteners</t>
-  </si>
-  <si>
-    <t>Minerallac</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>0.90</t>
   </si>
   <si>
-    <t>15</t>
-  </si>
-  <si>
     <t>44</t>
   </si>
   <si>
@@ -544,24 +400,9 @@
     <t>12 AWG THHN Copper Wire 500 ft spool</t>
   </si>
   <si>
-    <t>Wire</t>
-  </si>
-  <si>
-    <t>Southwire</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ft</t>
-  </si>
-  <si>
     <t>0.27</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
     <t>47</t>
   </si>
   <si>
@@ -577,27 +418,9 @@
     <t>1 in EMT Conduit 10 ft</t>
   </si>
   <si>
-    <t>Conduit</t>
-  </si>
-  <si>
-    <t>Allied Tube</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>stick</t>
-  </si>
-  <si>
     <t>10.80</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>880000001017</t>
   </si>
   <si>
@@ -610,27 +433,9 @@
     <t>EMT Set-Screw Connector #7</t>
   </si>
   <si>
-    <t>Fittings</t>
-  </si>
-  <si>
-    <t>Bridgeport</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>1.42</t>
   </si>
   <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>880000001018</t>
   </si>
   <si>
@@ -643,27 +448,9 @@
     <t>50A 1-pole QO Plug-On Breaker</t>
   </si>
   <si>
-    <t>Breakers</t>
-  </si>
-  <si>
-    <t>Square D</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>14.89</t>
   </si>
   <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>880000001019</t>
   </si>
   <si>
@@ -676,27 +463,9 @@
     <t>Steel Device Box #9</t>
   </si>
   <si>
-    <t>Boxes</t>
-  </si>
-  <si>
-    <t>Raco</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>3.39</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
     <t>880000001020</t>
   </si>
   <si>
@@ -709,27 +478,9 @@
     <t>LED Flat Panel #10</t>
   </si>
   <si>
-    <t>Lighting</t>
-  </si>
-  <si>
-    <t>Lithonia</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>59.54</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
     <t>880000001021</t>
   </si>
   <si>
@@ -742,27 +493,9 @@
     <t>Decorator Receptacle #11</t>
   </si>
   <si>
-    <t>Devices</t>
-  </si>
-  <si>
-    <t>Leviton</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>4.23</t>
   </si>
   <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
     <t>880000001022</t>
   </si>
   <si>
@@ -775,27 +508,9 @@
     <t>Strut Strap #12</t>
   </si>
   <si>
-    <t>Fasteners</t>
-  </si>
-  <si>
-    <t>Minerallac</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>0.85</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
     <t>880000001023</t>
   </si>
   <si>
@@ -808,27 +523,9 @@
     <t>6 AWG THHN Copper Wire 500 ft spool</t>
   </si>
   <si>
-    <t>Wire</t>
-  </si>
-  <si>
-    <t>Southwire</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ft</t>
-  </si>
-  <si>
     <t>0.26</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
     <t>880000001024</t>
   </si>
   <si>
@@ -841,27 +538,9 @@
     <t>1/2 in EMT Conduit 10 ft</t>
   </si>
   <si>
-    <t>Conduit</t>
-  </si>
-  <si>
-    <t>Allied Tube</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>stick</t>
-  </si>
-  <si>
     <t>10.29</t>
   </si>
   <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
     <t>880000001025</t>
   </si>
   <si>
@@ -871,30 +550,9 @@
     <t>F-01-026</t>
   </si>
   <si>
-    <t>EMT Set-Screw Connector #3</t>
-  </si>
-  <si>
-    <t>Fittings</t>
-  </si>
-  <si>
-    <t>Bridgeport</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>2.27</t>
   </si>
   <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
     <t>880000001026</t>
   </si>
   <si>
@@ -907,27 +565,9 @@
     <t>30A 1-pole QO Plug-On Breaker</t>
   </si>
   <si>
-    <t>Breakers</t>
-  </si>
-  <si>
-    <t>Square D</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>13.85</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
     <t>880000001027</t>
   </si>
   <si>
@@ -937,30 +577,9 @@
     <t>B-01-028</t>
   </si>
   <si>
-    <t>Steel Device Box #5</t>
-  </si>
-  <si>
-    <t>Boxes</t>
-  </si>
-  <si>
-    <t>Raco</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>3.17</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
     <t>880000001028</t>
   </si>
   <si>
@@ -970,30 +589,9 @@
     <t>L-01-029</t>
   </si>
   <si>
-    <t>LED Flat Panel #6</t>
-  </si>
-  <si>
-    <t>Lighting</t>
-  </si>
-  <si>
-    <t>Lithonia</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>55.89</t>
   </si>
   <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
     <t>880000001029</t>
   </si>
   <si>
@@ -1003,30 +601,9 @@
     <t>D-01-030</t>
   </si>
   <si>
-    <t>Decorator Receptacle #7</t>
-  </si>
-  <si>
-    <t>Devices</t>
-  </si>
-  <si>
-    <t>Leviton</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>3.98</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
     <t>880000001030</t>
   </si>
   <si>
@@ -1036,30 +613,9 @@
     <t>F-01-031</t>
   </si>
   <si>
-    <t>Strut Strap #8</t>
-  </si>
-  <si>
-    <t>Fasteners</t>
-  </si>
-  <si>
-    <t>Minerallac</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>0.81</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
     <t>880000001031</t>
   </si>
   <si>
@@ -1072,27 +628,9 @@
     <t>10 AWG THHN Copper Wire 500 ft spool</t>
   </si>
   <si>
-    <t>Wire</t>
-  </si>
-  <si>
-    <t>Southwire</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ft</t>
-  </si>
-  <si>
     <t>0.25</t>
   </si>
   <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
     <t>880000001032</t>
   </si>
   <si>
@@ -1105,27 +643,9 @@
     <t>1-1/4 in EMT Conduit 10 ft</t>
   </si>
   <si>
-    <t>Conduit</t>
-  </si>
-  <si>
-    <t>Allied Tube</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>stick</t>
-  </si>
-  <si>
     <t>9.79</t>
   </si>
   <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>880000001033</t>
   </si>
   <si>
@@ -1135,30 +655,9 @@
     <t>F-01-034</t>
   </si>
   <si>
-    <t>EMT Set-Screw Connector #11</t>
-  </si>
-  <si>
-    <t>Fittings</t>
-  </si>
-  <si>
-    <t>Bridgeport</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>2.17</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>880000001034</t>
   </si>
   <si>
@@ -1171,27 +670,9 @@
     <t>15A 1-pole QO Plug-On Breaker</t>
   </si>
   <si>
-    <t>Breakers</t>
-  </si>
-  <si>
-    <t>Square D</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>22.16</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>880000001035</t>
   </si>
   <si>
@@ -1201,28 +682,7 @@
     <t>B-01-036</t>
   </si>
   <si>
-    <t>Steel Device Box #1</t>
-  </si>
-  <si>
-    <t>Boxes</t>
-  </si>
-  <si>
-    <t>Raco</t>
-  </si>
-  <si>
-    <t>Codale Branch Quote</t>
-  </si>
-  <si>
-    <t>ea</t>
-  </si>
-  <si>
     <t>2.95</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>11</t>
   </si>
   <si>
     <t>880000001036</t>
@@ -1279,25 +739,25 @@
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>365</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>366</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>368</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
         <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s">
-        <v>371</v>
+        <v>19</v>
       </c>
       <c r="J2" t="s">
         <v>20</v>
@@ -1311,1224 +771,1224 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>287</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>376</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>377</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F3" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
         <v>28</v>
       </c>
-      <c r="H3" t="s">
-        <v>337</v>
-      </c>
       <c r="I3" t="s">
-        <v>382</v>
+        <v>29</v>
       </c>
       <c r="J3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" t="s">
         <v>31</v>
-      </c>
-      <c r="K3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="C4" t="s">
-        <v>387</v>
-      </c>
       <c r="D4" t="s">
-        <v>388</v>
+        <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" t="s">
         <v>39</v>
       </c>
-      <c r="H4" t="s">
-        <v>348</v>
-      </c>
-      <c r="I4" t="s">
-        <v>393</v>
-      </c>
-      <c r="J4" t="s">
-        <v>42</v>
-      </c>
       <c r="K4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" t="s">
-        <v>309</v>
-      </c>
-      <c r="C5" t="s">
-        <v>398</v>
-      </c>
-      <c r="D5" t="s">
-        <v>399</v>
-      </c>
       <c r="E5" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H5" t="s">
-        <v>359</v>
+        <v>46</v>
       </c>
       <c r="I5" t="s">
-        <v>404</v>
+        <v>47</v>
       </c>
       <c r="J5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="K5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" t="s">
         <v>55</v>
       </c>
-      <c r="B6" t="s">
-        <v>320</v>
-      </c>
-      <c r="C6" t="s">
-        <v>321</v>
-      </c>
-      <c r="D6" t="s">
-        <v>322</v>
-      </c>
-      <c r="E6" t="s">
-        <v>400</v>
-      </c>
-      <c r="F6" t="s">
-        <v>401</v>
-      </c>
-      <c r="G6" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" t="s">
-        <v>370</v>
-      </c>
       <c r="I6" t="s">
-        <v>239</v>
+        <v>56</v>
       </c>
       <c r="J6" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="K6" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" t="s">
+        <v>65</v>
+      </c>
+      <c r="J7" t="s">
         <v>66</v>
       </c>
-      <c r="B7" t="s">
-        <v>331</v>
-      </c>
-      <c r="C7" t="s">
-        <v>332</v>
-      </c>
-      <c r="D7" t="s">
-        <v>333</v>
-      </c>
-      <c r="E7" t="s">
-        <v>400</v>
-      </c>
-      <c r="F7" t="s">
-        <v>401</v>
-      </c>
-      <c r="G7" t="s">
-        <v>72</v>
-      </c>
-      <c r="H7" t="s">
-        <v>381</v>
-      </c>
-      <c r="I7" t="s">
-        <v>250</v>
-      </c>
-      <c r="J7" t="s">
-        <v>75</v>
-      </c>
       <c r="K7" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>342</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>343</v>
+        <v>70</v>
       </c>
       <c r="D8" t="s">
-        <v>344</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H8" t="s">
-        <v>392</v>
+        <v>73</v>
       </c>
       <c r="I8" t="s">
-        <v>261</v>
+        <v>74</v>
       </c>
       <c r="J8" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="K8" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="C9" t="s">
-        <v>354</v>
+        <v>79</v>
       </c>
       <c r="D9" t="s">
-        <v>355</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>357</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="H9" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="I9" t="s">
-        <v>272</v>
+        <v>83</v>
       </c>
       <c r="J9" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="K9" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="C10" t="s">
-        <v>365</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>366</v>
+        <v>14</v>
       </c>
       <c r="E10" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F10" t="s">
-        <v>368</v>
+        <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="H10" t="s">
-        <v>337</v>
+        <v>28</v>
       </c>
       <c r="I10" t="s">
-        <v>283</v>
+        <v>89</v>
       </c>
       <c r="J10" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="K10" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="B11" t="s">
-        <v>375</v>
+        <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>376</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>377</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F11" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="H11" t="s">
-        <v>348</v>
+        <v>37</v>
       </c>
       <c r="I11" t="s">
-        <v>294</v>
+        <v>95</v>
       </c>
       <c r="J11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="K11" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="B12" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>388</v>
+        <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F12" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="H12" t="s">
-        <v>359</v>
+        <v>46</v>
       </c>
       <c r="I12" t="s">
-        <v>305</v>
+        <v>101</v>
       </c>
       <c r="J12" t="s">
-        <v>130</v>
+        <v>102</v>
       </c>
       <c r="K12" t="s">
-        <v>131</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="B13" t="s">
-        <v>397</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
-        <v>398</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>399</v>
+        <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F13" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G13" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="H13" t="s">
-        <v>370</v>
+        <v>55</v>
       </c>
       <c r="I13" t="s">
-        <v>316</v>
+        <v>107</v>
       </c>
       <c r="J13" t="s">
-        <v>141</v>
+        <v>108</v>
       </c>
       <c r="K13" t="s">
-        <v>142</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>143</v>
+        <v>110</v>
       </c>
       <c r="B14" t="s">
-        <v>144</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
-        <v>321</v>
+        <v>52</v>
       </c>
       <c r="D14" t="s">
-        <v>322</v>
+        <v>53</v>
       </c>
       <c r="E14" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G14" t="s">
-        <v>149</v>
+        <v>112</v>
       </c>
       <c r="H14" t="s">
-        <v>381</v>
+        <v>64</v>
       </c>
       <c r="I14" t="s">
-        <v>327</v>
+        <v>113</v>
       </c>
       <c r="J14" t="s">
-        <v>152</v>
+        <v>114</v>
       </c>
       <c r="K14" t="s">
-        <v>153</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>154</v>
+        <v>116</v>
       </c>
       <c r="B15" t="s">
-        <v>155</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
-        <v>332</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>333</v>
+        <v>62</v>
       </c>
       <c r="E15" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F15" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G15" t="s">
-        <v>160</v>
+        <v>118</v>
       </c>
       <c r="H15" t="s">
-        <v>392</v>
+        <v>73</v>
       </c>
       <c r="I15" t="s">
-        <v>338</v>
+        <v>119</v>
       </c>
       <c r="J15" t="s">
-        <v>163</v>
+        <v>120</v>
       </c>
       <c r="K15" t="s">
-        <v>164</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="B16" t="s">
-        <v>166</v>
+        <v>123</v>
       </c>
       <c r="C16" t="s">
-        <v>343</v>
+        <v>70</v>
       </c>
       <c r="D16" t="s">
-        <v>344</v>
+        <v>71</v>
       </c>
       <c r="E16" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F16" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G16" t="s">
-        <v>171</v>
+        <v>124</v>
       </c>
       <c r="H16" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="I16" t="s">
-        <v>349</v>
+        <v>125</v>
       </c>
       <c r="J16" t="s">
-        <v>174</v>
+        <v>126</v>
       </c>
       <c r="K16" t="s">
-        <v>175</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>176</v>
+        <v>128</v>
       </c>
       <c r="B17" t="s">
-        <v>177</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>354</v>
+        <v>79</v>
       </c>
       <c r="D17" t="s">
-        <v>355</v>
+        <v>80</v>
       </c>
       <c r="E17" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F17" t="s">
-        <v>357</v>
+        <v>81</v>
       </c>
       <c r="G17" t="s">
-        <v>182</v>
+        <v>130</v>
       </c>
       <c r="H17" t="s">
-        <v>337</v>
+        <v>28</v>
       </c>
       <c r="I17" t="s">
-        <v>360</v>
+        <v>131</v>
       </c>
       <c r="J17" t="s">
-        <v>185</v>
+        <v>132</v>
       </c>
       <c r="K17" t="s">
-        <v>186</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>187</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>188</v>
+        <v>135</v>
       </c>
       <c r="C18" t="s">
-        <v>365</v>
+        <v>13</v>
       </c>
       <c r="D18" t="s">
-        <v>366</v>
+        <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F18" t="s">
-        <v>368</v>
+        <v>16</v>
       </c>
       <c r="G18" t="s">
-        <v>193</v>
+        <v>136</v>
       </c>
       <c r="H18" t="s">
-        <v>348</v>
+        <v>37</v>
       </c>
       <c r="I18" t="s">
-        <v>371</v>
+        <v>19</v>
       </c>
       <c r="J18" t="s">
-        <v>196</v>
+        <v>137</v>
       </c>
       <c r="K18" t="s">
-        <v>197</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>198</v>
+        <v>139</v>
       </c>
       <c r="B19" t="s">
-        <v>199</v>
+        <v>140</v>
       </c>
       <c r="C19" t="s">
-        <v>376</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
-        <v>377</v>
+        <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F19" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G19" t="s">
-        <v>204</v>
+        <v>141</v>
       </c>
       <c r="H19" t="s">
-        <v>359</v>
+        <v>46</v>
       </c>
       <c r="I19" t="s">
-        <v>382</v>
+        <v>29</v>
       </c>
       <c r="J19" t="s">
-        <v>207</v>
+        <v>142</v>
       </c>
       <c r="K19" t="s">
-        <v>208</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>209</v>
+        <v>144</v>
       </c>
       <c r="B20" t="s">
-        <v>210</v>
+        <v>145</v>
       </c>
       <c r="C20" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
-        <v>388</v>
+        <v>35</v>
       </c>
       <c r="E20" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G20" t="s">
-        <v>215</v>
+        <v>146</v>
       </c>
       <c r="H20" t="s">
-        <v>370</v>
+        <v>55</v>
       </c>
       <c r="I20" t="s">
-        <v>393</v>
+        <v>38</v>
       </c>
       <c r="J20" t="s">
-        <v>218</v>
+        <v>147</v>
       </c>
       <c r="K20" t="s">
-        <v>219</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>220</v>
+        <v>149</v>
       </c>
       <c r="B21" t="s">
-        <v>221</v>
+        <v>150</v>
       </c>
       <c r="C21" t="s">
-        <v>398</v>
+        <v>43</v>
       </c>
       <c r="D21" t="s">
-        <v>399</v>
+        <v>44</v>
       </c>
       <c r="E21" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F21" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G21" t="s">
-        <v>226</v>
+        <v>151</v>
       </c>
       <c r="H21" t="s">
-        <v>381</v>
+        <v>64</v>
       </c>
       <c r="I21" t="s">
-        <v>404</v>
+        <v>47</v>
       </c>
       <c r="J21" t="s">
-        <v>229</v>
+        <v>152</v>
       </c>
       <c r="K21" t="s">
-        <v>230</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>231</v>
+        <v>154</v>
       </c>
       <c r="B22" t="s">
-        <v>232</v>
+        <v>155</v>
       </c>
       <c r="C22" t="s">
-        <v>321</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>322</v>
+        <v>53</v>
       </c>
       <c r="E22" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F22" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G22" t="s">
-        <v>237</v>
+        <v>156</v>
       </c>
       <c r="H22" t="s">
-        <v>392</v>
+        <v>73</v>
       </c>
       <c r="I22" t="s">
-        <v>239</v>
+        <v>56</v>
       </c>
       <c r="J22" t="s">
-        <v>240</v>
+        <v>157</v>
       </c>
       <c r="K22" t="s">
-        <v>241</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>242</v>
+        <v>159</v>
       </c>
       <c r="B23" t="s">
-        <v>243</v>
+        <v>160</v>
       </c>
       <c r="C23" t="s">
-        <v>332</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>333</v>
+        <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F23" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G23" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="H23" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="I23" t="s">
-        <v>250</v>
+        <v>65</v>
       </c>
       <c r="J23" t="s">
-        <v>251</v>
+        <v>162</v>
       </c>
       <c r="K23" t="s">
-        <v>252</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>253</v>
+        <v>164</v>
       </c>
       <c r="B24" t="s">
-        <v>254</v>
+        <v>165</v>
       </c>
       <c r="C24" t="s">
-        <v>343</v>
+        <v>70</v>
       </c>
       <c r="D24" t="s">
-        <v>344</v>
+        <v>71</v>
       </c>
       <c r="E24" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F24" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G24" t="s">
-        <v>259</v>
+        <v>166</v>
       </c>
       <c r="H24" t="s">
-        <v>337</v>
+        <v>28</v>
       </c>
       <c r="I24" t="s">
-        <v>261</v>
+        <v>74</v>
       </c>
       <c r="J24" t="s">
-        <v>262</v>
+        <v>167</v>
       </c>
       <c r="K24" t="s">
-        <v>263</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>264</v>
+        <v>169</v>
       </c>
       <c r="B25" t="s">
-        <v>265</v>
+        <v>170</v>
       </c>
       <c r="C25" t="s">
-        <v>354</v>
+        <v>79</v>
       </c>
       <c r="D25" t="s">
-        <v>355</v>
+        <v>80</v>
       </c>
       <c r="E25" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F25" t="s">
-        <v>357</v>
+        <v>81</v>
       </c>
       <c r="G25" t="s">
-        <v>270</v>
+        <v>171</v>
       </c>
       <c r="H25" t="s">
-        <v>348</v>
+        <v>37</v>
       </c>
       <c r="I25" t="s">
-        <v>272</v>
+        <v>83</v>
       </c>
       <c r="J25" t="s">
-        <v>273</v>
+        <v>172</v>
       </c>
       <c r="K25" t="s">
-        <v>274</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>275</v>
+        <v>174</v>
       </c>
       <c r="B26" t="s">
-        <v>276</v>
+        <v>175</v>
       </c>
       <c r="C26" t="s">
-        <v>365</v>
+        <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>366</v>
+        <v>14</v>
       </c>
       <c r="E26" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F26" t="s">
-        <v>368</v>
+        <v>16</v>
       </c>
       <c r="G26" t="s">
-        <v>281</v>
+        <v>176</v>
       </c>
       <c r="H26" t="s">
-        <v>359</v>
+        <v>46</v>
       </c>
       <c r="I26" t="s">
-        <v>283</v>
+        <v>89</v>
       </c>
       <c r="J26" t="s">
-        <v>284</v>
+        <v>177</v>
       </c>
       <c r="K26" t="s">
-        <v>285</v>
+        <v>178</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>286</v>
+        <v>179</v>
       </c>
       <c r="B27" t="s">
-        <v>287</v>
+        <v>23</v>
       </c>
       <c r="C27" t="s">
-        <v>376</v>
+        <v>24</v>
       </c>
       <c r="D27" t="s">
-        <v>377</v>
+        <v>25</v>
       </c>
       <c r="E27" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F27" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G27" t="s">
-        <v>292</v>
+        <v>180</v>
       </c>
       <c r="H27" t="s">
-        <v>370</v>
+        <v>55</v>
       </c>
       <c r="I27" t="s">
-        <v>294</v>
+        <v>95</v>
       </c>
       <c r="J27" t="s">
-        <v>295</v>
+        <v>181</v>
       </c>
       <c r="K27" t="s">
-        <v>296</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>297</v>
+        <v>183</v>
       </c>
       <c r="B28" t="s">
-        <v>298</v>
+        <v>184</v>
       </c>
       <c r="C28" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="D28" t="s">
-        <v>388</v>
+        <v>35</v>
       </c>
       <c r="E28" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F28" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G28" t="s">
-        <v>303</v>
+        <v>185</v>
       </c>
       <c r="H28" t="s">
-        <v>381</v>
+        <v>64</v>
       </c>
       <c r="I28" t="s">
-        <v>305</v>
+        <v>101</v>
       </c>
       <c r="J28" t="s">
-        <v>306</v>
+        <v>186</v>
       </c>
       <c r="K28" t="s">
-        <v>307</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>308</v>
+        <v>188</v>
       </c>
       <c r="B29" t="s">
-        <v>309</v>
+        <v>42</v>
       </c>
       <c r="C29" t="s">
-        <v>398</v>
+        <v>43</v>
       </c>
       <c r="D29" t="s">
-        <v>399</v>
+        <v>44</v>
       </c>
       <c r="E29" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F29" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G29" t="s">
-        <v>314</v>
+        <v>189</v>
       </c>
       <c r="H29" t="s">
-        <v>392</v>
+        <v>73</v>
       </c>
       <c r="I29" t="s">
-        <v>316</v>
+        <v>107</v>
       </c>
       <c r="J29" t="s">
-        <v>317</v>
+        <v>190</v>
       </c>
       <c r="K29" t="s">
-        <v>318</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>319</v>
+        <v>192</v>
       </c>
       <c r="B30" t="s">
-        <v>320</v>
+        <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>321</v>
+        <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>322</v>
+        <v>53</v>
       </c>
       <c r="E30" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F30" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G30" t="s">
-        <v>325</v>
+        <v>193</v>
       </c>
       <c r="H30" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="I30" t="s">
-        <v>327</v>
+        <v>113</v>
       </c>
       <c r="J30" t="s">
-        <v>328</v>
+        <v>194</v>
       </c>
       <c r="K30" t="s">
-        <v>329</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>330</v>
+        <v>196</v>
       </c>
       <c r="B31" t="s">
-        <v>331</v>
+        <v>60</v>
       </c>
       <c r="C31" t="s">
-        <v>332</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>333</v>
+        <v>62</v>
       </c>
       <c r="E31" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F31" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G31" t="s">
-        <v>336</v>
+        <v>197</v>
       </c>
       <c r="H31" t="s">
-        <v>337</v>
+        <v>28</v>
       </c>
       <c r="I31" t="s">
-        <v>338</v>
+        <v>119</v>
       </c>
       <c r="J31" t="s">
-        <v>339</v>
+        <v>198</v>
       </c>
       <c r="K31" t="s">
-        <v>340</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>341</v>
+        <v>200</v>
       </c>
       <c r="B32" t="s">
-        <v>342</v>
+        <v>69</v>
       </c>
       <c r="C32" t="s">
-        <v>343</v>
+        <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>344</v>
+        <v>71</v>
       </c>
       <c r="E32" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F32" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G32" t="s">
-        <v>347</v>
+        <v>201</v>
       </c>
       <c r="H32" t="s">
-        <v>348</v>
+        <v>37</v>
       </c>
       <c r="I32" t="s">
-        <v>349</v>
+        <v>125</v>
       </c>
       <c r="J32" t="s">
-        <v>350</v>
+        <v>202</v>
       </c>
       <c r="K32" t="s">
-        <v>351</v>
+        <v>203</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>352</v>
+        <v>204</v>
       </c>
       <c r="B33" t="s">
-        <v>353</v>
+        <v>205</v>
       </c>
       <c r="C33" t="s">
-        <v>354</v>
+        <v>79</v>
       </c>
       <c r="D33" t="s">
-        <v>355</v>
+        <v>80</v>
       </c>
       <c r="E33" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F33" t="s">
-        <v>357</v>
+        <v>81</v>
       </c>
       <c r="G33" t="s">
-        <v>358</v>
+        <v>206</v>
       </c>
       <c r="H33" t="s">
-        <v>359</v>
+        <v>46</v>
       </c>
       <c r="I33" t="s">
-        <v>360</v>
+        <v>131</v>
       </c>
       <c r="J33" t="s">
-        <v>361</v>
+        <v>207</v>
       </c>
       <c r="K33" t="s">
-        <v>362</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>363</v>
+        <v>209</v>
       </c>
       <c r="B34" t="s">
-        <v>364</v>
+        <v>210</v>
       </c>
       <c r="C34" t="s">
-        <v>365</v>
+        <v>13</v>
       </c>
       <c r="D34" t="s">
-        <v>366</v>
+        <v>14</v>
       </c>
       <c r="E34" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F34" t="s">
-        <v>368</v>
+        <v>16</v>
       </c>
       <c r="G34" t="s">
-        <v>369</v>
+        <v>211</v>
       </c>
       <c r="H34" t="s">
-        <v>370</v>
+        <v>55</v>
       </c>
       <c r="I34" t="s">
-        <v>371</v>
+        <v>19</v>
       </c>
       <c r="J34" t="s">
-        <v>372</v>
+        <v>212</v>
       </c>
       <c r="K34" t="s">
-        <v>373</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>374</v>
+        <v>214</v>
       </c>
       <c r="B35" t="s">
-        <v>375</v>
+        <v>93</v>
       </c>
       <c r="C35" t="s">
-        <v>376</v>
+        <v>24</v>
       </c>
       <c r="D35" t="s">
-        <v>377</v>
+        <v>25</v>
       </c>
       <c r="E35" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F35" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G35" t="s">
-        <v>380</v>
+        <v>215</v>
       </c>
       <c r="H35" t="s">
-        <v>381</v>
+        <v>64</v>
       </c>
       <c r="I35" t="s">
-        <v>382</v>
+        <v>29</v>
       </c>
       <c r="J35" t="s">
-        <v>383</v>
+        <v>216</v>
       </c>
       <c r="K35" t="s">
-        <v>384</v>
+        <v>217</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>385</v>
+        <v>218</v>
       </c>
       <c r="B36" t="s">
-        <v>386</v>
+        <v>219</v>
       </c>
       <c r="C36" t="s">
-        <v>387</v>
+        <v>34</v>
       </c>
       <c r="D36" t="s">
-        <v>388</v>
+        <v>35</v>
       </c>
       <c r="E36" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F36" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G36" t="s">
-        <v>391</v>
+        <v>220</v>
       </c>
       <c r="H36" t="s">
-        <v>392</v>
+        <v>73</v>
       </c>
       <c r="I36" t="s">
-        <v>393</v>
+        <v>38</v>
       </c>
       <c r="J36" t="s">
-        <v>394</v>
+        <v>221</v>
       </c>
       <c r="K36" t="s">
-        <v>395</v>
+        <v>222</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>396</v>
+        <v>223</v>
       </c>
       <c r="B37" t="s">
-        <v>397</v>
+        <v>105</v>
       </c>
       <c r="C37" t="s">
-        <v>398</v>
+        <v>43</v>
       </c>
       <c r="D37" t="s">
-        <v>399</v>
+        <v>44</v>
       </c>
       <c r="E37" t="s">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="F37" t="s">
-        <v>401</v>
+        <v>26</v>
       </c>
       <c r="G37" t="s">
-        <v>402</v>
+        <v>224</v>
       </c>
       <c r="H37" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="I37" t="s">
-        <v>404</v>
+        <v>47</v>
       </c>
       <c r="J37" t="s">
-        <v>405</v>
+        <v>225</v>
       </c>
       <c r="K37" t="s">
-        <v>406</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>